<commit_message>
Inspector import: blank DisplayType, defaults for read-only outputs
DisplayType is a restricted picklist in the org (Dropdown rejected); visible
read-only attributes require a DefaultValue. Airlite2 workbook rebuilt with a
retry tab holding the 28 failed ProductClassificationAttr rows.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D8YckfAx7oSp47X8zmY1mN
</commit_message>
<xml_diff>
--- a/OneDrive_2026-09-29/Claude RCA Product/10-airlite2-product-template/Airlite2_RCA_Import_Inspector.xlsx
+++ b/OneDrive_2026-09-29/Claude RCA Product/10-airlite2-product-template/Airlite2_RCA_Import_Inspector.xlsx
@@ -16,9 +16,10 @@
     <sheet name="06 Product2" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="07 AttributeCategoryAttr" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="08 ProductClassificationAttr" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="09 ProductCategoryProduct" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="10 PricebookEntry" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="11 Attribute_Pricing__c" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="08 RETRY (failed rows)" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="09 ProductCategoryProduct" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="10 PricebookEntry" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="11 Attribute_Pricing__c" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -650,7 +651,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Calculated outputs are IsReadOnly = true. DisplayType is only set (Dropdown) for picklists.</t>
+          <t>Calculated outputs are IsReadOnly = true with a default (0 for numbers, X for text) – required for visible read-only attributes; the constraint model overwrites them. DisplayType left blank (restricted picklist – 'Dropdown' is rejected; blank uses the attribute type's default).</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
@@ -760,6 +761,1542 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="54" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="46" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>AttributeCategory:AttributeCategory:Code</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>IsPriceImpacting</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>IsHidden</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>IsReadOnly</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>IsRequired</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>DisplayType</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>AttributeDefinition:AttributeDefinition:Code</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>DefaultValue</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>ProductClassification:ProductClassification:Code</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification_AIR_Version2</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Device_Configuration</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="n"/>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>AIR_Version2</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>1E</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification_AIR_Width2</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Device_Configuration</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="n"/>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>AIR_Width2</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="n"/>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification_AIR_Length2</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Device_Configuration</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="n"/>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>AIR_Length2</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification_AIR_Insulation2</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Device_Configuration</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="n"/>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>AIR_Insulation2</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification_AIR_Louvre2</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Filling</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="n"/>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>AIR_Louvre2</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="n"/>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification_AIR_Controls2</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Control_and_Drive</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="n"/>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>AIR_Controls2</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="n"/>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification_AIR_ThermalRelease2</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Control_and_Drive</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="n"/>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>AIR_ThermalRelease2</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>FX</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification_AIR_ControlBracket2</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Control_and_Drive</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="n"/>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>AIR_ControlBracket2</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="n"/>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification_AIR_BaseDesign2</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Base_and_Flange</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="n"/>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>AIR_BaseDesign2</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="n"/>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification_AIR_FlangeType2</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Base_and_Flange</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="n"/>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>AIR_FlangeType2</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>N5</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification_AIR_Coating2</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Finish</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="n"/>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>AIR_Coating2</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>130</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification_AIR_CoatingThickness2</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Finish</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="n"/>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>AIR_CoatingThickness2</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification_AIR_InstallationType2</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Installation</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="n"/>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>AIR_InstallationType2</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="n"/>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>160</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification_AIR_WindBaffle2</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Installation</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="n"/>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>AIR_WindBaffle2</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="n"/>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>180</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification_AIR_Delivery2</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Options</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="n"/>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>AIR_Delivery2</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>190</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification_AIR_AmbientTemp2</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Loads_and_Pressure</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="n"/>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AmbientTemp2</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>T(-15)</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification_AIR_CylinderType2</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Calculated_Outputs</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="n"/>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>AIR_CylinderType2</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification_AIR_CO2Bottle2</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Calculated_Outputs</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="n"/>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>AIR_CO2Bottle2</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>310</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification_AIR_StandbyReservoir2</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Calculated_Outputs</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="n"/>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>AIR_StandbyReservoir2</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>320</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification_AIR_ElectricDrive2</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Calculated_Outputs</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="n"/>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>AIR_ElectricDrive2</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="inlineStr">
+        <is>
+          <t>330</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification_AIR_WindSuctionLoad2</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Calculated_Outputs</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="n"/>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>AIR_WindSuctionLoad2</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>340</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification_AIR_GeomAreaAv2</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Calculated_Outputs</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="n"/>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>AIR_GeomAreaAv2</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification</t>
+        </is>
+      </c>
+      <c r="K23" s="3" t="inlineStr">
+        <is>
+          <t>350</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification_AIR_AeroAreaAa2</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Calculated_Outputs</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="n"/>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AeroAreaAa2</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>360</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification_AIR_UValue2</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Calculated_Outputs</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="n"/>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>AIR_UValue2</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification</t>
+        </is>
+      </c>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
+          <t>370</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification_AIR_LouvreWeight2</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Calculated_Outputs</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="n"/>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>AIR_LouvreWeight2</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>380</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification_AIR_TotalWeight2</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Calculated_Outputs</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="n"/>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>AIR_TotalWeight2</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>390</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification_AIR_MaxSLCylinder2</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Calculated_Outputs</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="n"/>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>AIR_MaxSLCylinder2</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification</t>
+        </is>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification_AIR_MaxSLMotor2</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Calculated_Outputs</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="n"/>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>AIR_MaxSLMotor2</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>AIR_AIR2_ProductClassification</t>
+        </is>
+      </c>
+      <c r="K29" s="3" t="inlineStr">
+        <is>
+          <t>410</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -801,7 +2338,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -876,7 +2413,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10258,11 +11795,7 @@
           <t>false</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>Dropdown</t>
-        </is>
-      </c>
+      <c r="G2" s="3" t="inlineStr"/>
       <c r="H2" s="3" t="inlineStr">
         <is>
           <t>AIR_Version2</t>
@@ -10315,11 +11848,7 @@
           <t>false</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Dropdown</t>
-        </is>
-      </c>
+      <c r="G3" s="3" t="inlineStr"/>
       <c r="H3" s="3" t="inlineStr">
         <is>
           <t>AIR_Width2</t>
@@ -10368,11 +11897,7 @@
           <t>false</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Dropdown</t>
-        </is>
-      </c>
+      <c r="G4" s="3" t="inlineStr"/>
       <c r="H4" s="3" t="inlineStr">
         <is>
           <t>AIR_Length2</t>
@@ -10519,11 +12044,7 @@
           <t>false</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>Dropdown</t>
-        </is>
-      </c>
+      <c r="G7" s="3" t="inlineStr"/>
       <c r="H7" s="3" t="inlineStr">
         <is>
           <t>AIR_Insulation2</t>
@@ -10576,11 +12097,7 @@
           <t>false</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>Dropdown</t>
-        </is>
-      </c>
+      <c r="G8" s="3" t="inlineStr"/>
       <c r="H8" s="3" t="inlineStr">
         <is>
           <t>AIR_Louvre2</t>
@@ -10629,11 +12146,7 @@
           <t>false</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>Dropdown</t>
-        </is>
-      </c>
+      <c r="G9" s="3" t="inlineStr"/>
       <c r="H9" s="3" t="inlineStr">
         <is>
           <t>AIR_Controls2</t>
@@ -10682,11 +12195,7 @@
           <t>false</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>Dropdown</t>
-        </is>
-      </c>
+      <c r="G10" s="3" t="inlineStr"/>
       <c r="H10" s="3" t="inlineStr">
         <is>
           <t>AIR_ThermalRelease2</t>
@@ -10739,11 +12248,7 @@
           <t>false</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>Dropdown</t>
-        </is>
-      </c>
+      <c r="G11" s="3" t="inlineStr"/>
       <c r="H11" s="3" t="inlineStr">
         <is>
           <t>AIR_ControlBracket2</t>
@@ -10792,11 +12297,7 @@
           <t>false</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>Dropdown</t>
-        </is>
-      </c>
+      <c r="G12" s="3" t="inlineStr"/>
       <c r="H12" s="3" t="inlineStr">
         <is>
           <t>AIR_BaseDesign2</t>
@@ -10845,11 +12346,7 @@
           <t>false</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>Dropdown</t>
-        </is>
-      </c>
+      <c r="G13" s="3" t="inlineStr"/>
       <c r="H13" s="3" t="inlineStr">
         <is>
           <t>AIR_FlangeType2</t>
@@ -10902,11 +12399,7 @@
           <t>false</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>Dropdown</t>
-        </is>
-      </c>
+      <c r="G14" s="3" t="inlineStr"/>
       <c r="H14" s="3" t="inlineStr">
         <is>
           <t>AIR_Coating2</t>
@@ -11008,11 +12501,7 @@
           <t>false</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>Dropdown</t>
-        </is>
-      </c>
+      <c r="G16" s="3" t="inlineStr"/>
       <c r="H16" s="3" t="inlineStr">
         <is>
           <t>AIR_CoatingThickness2</t>
@@ -11065,11 +12554,7 @@
           <t>false</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>Dropdown</t>
-        </is>
-      </c>
+      <c r="G17" s="3" t="inlineStr"/>
       <c r="H17" s="3" t="inlineStr">
         <is>
           <t>AIR_InstallationType2</t>
@@ -11167,11 +12652,7 @@
           <t>false</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>Dropdown</t>
-        </is>
-      </c>
+      <c r="G19" s="3" t="inlineStr"/>
       <c r="H19" s="3" t="inlineStr">
         <is>
           <t>AIR_WindBaffle2</t>
@@ -11220,11 +12701,7 @@
           <t>false</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>Dropdown</t>
-        </is>
-      </c>
+      <c r="G20" s="3" t="inlineStr"/>
       <c r="H20" s="3" t="inlineStr">
         <is>
           <t>AIR_Delivery2</t>
@@ -11375,11 +12852,7 @@
           <t>false</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>Dropdown</t>
-        </is>
-      </c>
+      <c r="G23" s="3" t="inlineStr"/>
       <c r="H23" s="3" t="inlineStr">
         <is>
           <t>AIR_AmbientTemp2</t>
@@ -11544,7 +13017,11 @@
           <t>AIR_CylinderType2</t>
         </is>
       </c>
-      <c r="I26" s="3" t="inlineStr"/>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
           <t>AIR_AIR2_ProductClassification</t>
@@ -11593,7 +13070,11 @@
           <t>AIR_CO2Bottle2</t>
         </is>
       </c>
-      <c r="I27" s="3" t="inlineStr"/>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
           <t>AIR_AIR2_ProductClassification</t>
@@ -11642,7 +13123,11 @@
           <t>AIR_StandbyReservoir2</t>
         </is>
       </c>
-      <c r="I28" s="3" t="inlineStr"/>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
           <t>AIR_AIR2_ProductClassification</t>
@@ -11691,7 +13176,11 @@
           <t>AIR_ElectricDrive2</t>
         </is>
       </c>
-      <c r="I29" s="3" t="inlineStr"/>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
           <t>AIR_AIR2_ProductClassification</t>
@@ -11740,7 +13229,11 @@
           <t>AIR_WindSuctionLoad2</t>
         </is>
       </c>
-      <c r="I30" s="3" t="inlineStr"/>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
           <t>AIR_AIR2_ProductClassification</t>
@@ -11789,7 +13282,11 @@
           <t>AIR_GeomAreaAv2</t>
         </is>
       </c>
-      <c r="I31" s="3" t="inlineStr"/>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
           <t>AIR_AIR2_ProductClassification</t>
@@ -11838,7 +13335,11 @@
           <t>AIR_AeroAreaAa2</t>
         </is>
       </c>
-      <c r="I32" s="3" t="inlineStr"/>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
           <t>AIR_AIR2_ProductClassification</t>
@@ -11887,7 +13388,11 @@
           <t>AIR_UValue2</t>
         </is>
       </c>
-      <c r="I33" s="3" t="inlineStr"/>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
           <t>AIR_AIR2_ProductClassification</t>
@@ -11936,7 +13441,11 @@
           <t>AIR_LouvreWeight2</t>
         </is>
       </c>
-      <c r="I34" s="3" t="inlineStr"/>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
           <t>AIR_AIR2_ProductClassification</t>
@@ -11985,7 +13494,11 @@
           <t>AIR_TotalWeight2</t>
         </is>
       </c>
-      <c r="I35" s="3" t="inlineStr"/>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
           <t>AIR_AIR2_ProductClassification</t>
@@ -12034,7 +13547,11 @@
           <t>AIR_MaxSLCylinder2</t>
         </is>
       </c>
-      <c r="I36" s="3" t="inlineStr"/>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
           <t>AIR_AIR2_ProductClassification</t>
@@ -12083,7 +13600,11 @@
           <t>AIR_MaxSLMotor2</t>
         </is>
       </c>
-      <c r="I37" s="3" t="inlineStr"/>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="J37" s="3" t="inlineStr">
         <is>
           <t>AIR_AIR2_ProductClassification</t>

</xml_diff>

<commit_message>
Import Steps: CML and TEST as labelled steps, not numbered like tabs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D8YckfAx7oSp47X8zmY1mN
</commit_message>
<xml_diff>
--- a/OneDrive_2026-09-29/Claude RCA Product/10-airlite2-product-template/Airlite2_RCA_Import_Inspector.xlsx
+++ b/OneDrive_2026-09-29/Claude RCA Product/10-airlite2-product-template/Airlite2_RCA_Import_Inspector.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -689,71 +689,109 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
+          <t>CML – Constraint model</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Constraint Builder</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr"/>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Not an Inspector import. Create the constraint model for the product, paste the .cml file, Validate, Activate.</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>TEST – Quote</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Quote</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Create a quote, add the product, configure. Check dropdowns, rules and calculated outputs.</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
           <t>10 PricebookEntry</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>Insert – LATER</t>
         </is>
       </c>
-      <c r="C11" s="2" t="n">
+      <c r="C13" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>Skip until the factory supplies prices. Standard Price Book entry first, then the KLAW price book.</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>Pricebook2Id:
 SELECT Id, Name, IsStandard FROM Pricebook2 WHERE IsActive = true</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>11 Attribute_Pricing__c</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Insert – LATER</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Skip until prices are known (see the template's Configurable Product Pricing tab).</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n"/>
-      <c r="B13" s="2" t="n"/>
-      <c r="C13" s="2" t="n"/>
-      <c r="D13" s="2" t="n"/>
-      <c r="E13" s="2" t="n"/>
-    </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t>11 Attribute_Pricing__c</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Insert – LATER</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Skip until prices are known (see the template's Configurable Product Pricing tab).</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n"/>
+      <c r="B15" s="2" t="n"/>
+      <c r="C15" s="2" t="n"/>
+      <c r="D15" s="2" t="n"/>
+      <c r="E15" s="2" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
           <t>How</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Salesforce Inspector Reloaded → Data Import. For each tab in order: pick the object, action Insert, copy the whole tab (incl. header row) and paste into the data box, check the field mapping, Run. Fix any red rows, re-run only those, then move to the next tab.</t>
         </is>
       </c>
-      <c r="C14" s="2" t="n"/>
-      <c r="D14" s="2" t="n"/>
-      <c r="E14" s="2" t="n"/>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Skill: constraint model steps CML-1..CML-6 + TEST in the import sequence
- build_inspector_import.py: --cml / --test; Import Steps tab lists 01-09,
  CML-1..CML-6 (check attributes, create, paste, link, validate, activate),
  TEST, then pricing 10-11.
- SKILL.md Phase 7 with the sequence table; definition of done updated.
- csv_import_reference.md and cml_syntax_rules.md: CML steps and Airlite lessons.
- Airlite2 workbook rebuilt with the new steps (08 RETRY tab kept).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D8YckfAx7oSp47X8zmY1mN
</commit_message>
<xml_diff>
--- a/OneDrive_2026-09-29/Claude RCA Product/10-airlite2-product-template/Airlite2_RCA_Import_Inspector.xlsx
+++ b/OneDrive_2026-09-29/Claude RCA Product/10-airlite2-product-template/Airlite2_RCA_Import_Inspector.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -689,37 +689,41 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>CML – Constraint model</t>
+          <t>CML-1 Check attributes</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Constraint Builder</t>
+          <t>Data Export</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr"/>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Not an Inspector import. Create the constraint model for the product, paste the .cml file, Validate, Activate.</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr"/>
+          <t>Before loading the model, every attribute named in the .cml must exist and be linked to the classification (tabs 02 and 08 fully succeeded). Expect all configurable + output attributes.</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>SELECT AttributeDefinition.Code, IsReadOnly, DefaultValue FROM ProductClassificationAttr WHERE ProductClassification.Code = 'AIR_AIR2_ProductClassification' ORDER BY Sequence</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>TEST – Quote</t>
+          <t>CML-2 Create model</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Quote</t>
+          <t>Constraint Builder</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr"/>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Create a quote, add the product, configure. Check dropdowns, rules and calculated outputs.</t>
+          <t>Not an Inspector import. App Launcher → Constraint Models → New. Name it after the product (e.g. AIR2 Constraint Model) and create / open its first version in the Constraint Builder.</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
@@ -727,71 +731,166 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
+          <t>CML-3 Paste CML</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Constraint Builder</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr"/>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Open the CML editor of that version, select all and replace with the full contents of Airlite2_ConstraintModel.cml. The file declares 'type AirliteAIR2 : LineItem'. Save.</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>CML-4 Link product</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Constraint Builder</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Associate the type AirliteAIR2 with product AIR2 (product / classification association in the model), so the model runs when AIR2 is configured.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>CML-5 Validate</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Constraint Builder</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr"/>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Validate / compile. On an error, note the message and line number – common causes are in references/cml_syntax_rules.md (unsupported annotation, string method, ROUND, decimal arithmetic → tree-node search limit). Fix the .cml, paste again, re-validate.</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>CML-6 Activate</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Constraint Builder</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Activate the version. Only one active version per model.</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>TEST – Quote</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Quote</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr"/>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Create a quote, add the product, configure. Check: every attribute shows, dropdown values are right, invalid combinations are blocked with the rule message, calculated outputs fill in. Reference configuration: AIR2, Width 1200, Length 2100, Installation A0, Wind baffle WM → Av 2.52 m², Aa 1.42 m²</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>10 PricebookEntry</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>Insert – LATER</t>
         </is>
       </c>
-      <c r="C13" s="2" t="n">
+      <c r="C18" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>Skip until the factory supplies prices. Standard Price Book entry first, then the KLAW price book.</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>Pricebook2Id:
 SELECT Id, Name, IsStandard FROM Pricebook2 WHERE IsActive = true</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>11 Attribute_Pricing__c</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>Insert – LATER</t>
         </is>
       </c>
-      <c r="C14" s="2" t="n">
+      <c r="C19" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>Skip until prices are known (see the template's Configurable Product Pricing tab).</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="n"/>
-      <c r="B15" s="2" t="n"/>
-      <c r="C15" s="2" t="n"/>
-      <c r="D15" s="2" t="n"/>
-      <c r="E15" s="2" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n"/>
+      <c r="B20" s="2" t="n"/>
+      <c r="C20" s="2" t="n"/>
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>How</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>Salesforce Inspector Reloaded → Data Import. For each tab in order: pick the object, action Insert, copy the whole tab (incl. header row) and paste into the data box, check the field mapping, Run. Fix any red rows, re-run only those, then move to the next tab.</t>
         </is>
       </c>
-      <c r="C16" s="2" t="n"/>
-      <c r="D16" s="2" t="n"/>
-      <c r="E16" s="2" t="n"/>
+      <c r="C21" s="2" t="n"/>
+      <c r="D21" s="2" t="n"/>
+      <c r="E21" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Skill: CML-4 association is required before activation
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D8YckfAx7oSp47X8zmY1mN
</commit_message>
<xml_diff>
--- a/OneDrive_2026-09-29/Claude RCA Product/10-airlite2-product-template/Airlite2_RCA_Import_Inspector.xlsx
+++ b/OneDrive_2026-09-29/Claude RCA Product/10-airlite2-product-template/Airlite2_RCA_Import_Inspector.xlsx
@@ -761,10 +761,19 @@
       <c r="C14" s="2" t="inlineStr"/>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Associate the type AirliteAIR2 with product AIR2 (product / classification association in the model), so the model runs when AIR2 is configured.</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr"/>
+          <t>REQUIRED before activation (else: 'We couldn't find any associations for constraint version …'). Associations tab → New: reference object = product AIR2, tag = AirliteAIR2 (exactly the CML type name), tag type = Type. No UI? Insert ExpressionSetConstraintObj with Inspector: ExpressionSetId, ReferenceObjectId (product Id), ConstraintModelTag = AirliteAIR2, ConstraintModelTagType = Type. Copy the pattern from a working model.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>How a working model (ECO) is linked:
+SELECT Id, ExpressionSet.Name, ReferenceObjectId, ReferenceObject.Name, ConstraintModelTag, ConstraintModelTagType FROM ExpressionSetConstraintObj WHERE ExpressionSet.Name LIKE '%ECO%'
+Model Id:
+SELECT Id, Name FROM ExpressionSet WHERE Name LIKE '%AIR2%'
+Product Id:
+SELECT Id, Name FROM Product2 WHERE ProductCode = 'AIR2'</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Skill: CML-4 association = ExpressionSetConstraintObj insert (confirmed)
Structure confirmed from the org's ECO association. Inspector workbook gets a
'CML-4 ExpressionSetConstraintObj' tab; Airlite2 tab pre-filled with the AIR2
constraint model Id.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D8YckfAx7oSp47X8zmY1mN
</commit_message>
<xml_diff>
--- a/OneDrive_2026-09-29/Claude RCA Product/10-airlite2-product-template/Airlite2_RCA_Import_Inspector.xlsx
+++ b/OneDrive_2026-09-29/Claude RCA Product/10-airlite2-product-template/Airlite2_RCA_Import_Inspector.xlsx
@@ -18,8 +18,9 @@
     <sheet name="08 ProductClassificationAttr" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="08 RETRY (failed rows)" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="09 ProductCategoryProduct" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="10 PricebookEntry" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="11 Attribute_Pricing__c" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="CML-4 ExpressionSetConstraintObj" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="10 PricebookEntry" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="11 Attribute_Pricing__c" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -761,14 +762,14 @@
       <c r="C14" s="2" t="inlineStr"/>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>REQUIRED before activation (else: 'We couldn't find any associations for constraint version …'). NOT 'New Type' (that only adds a CML type – Name + Parent type) and not 'Add Labels'. UNCONFIRMED route: copy a working model's association (query) and Insert ExpressionSetConstraintObj with Inspector: ExpressionSetId, ReferenceObjectId (product Id), ConstraintModelTag = AirliteAIR2, ConstraintModelTagType = Type. Copy the pattern from a working model.</t>
+          <t>REQUIRED before activation (else: 'We couldn't find any associations for constraint version 9QL…'). Not done in the Constraint Builder UI ('New Type' only adds a CML type; 'Add Labels' is unrelated). Inspector → Data Import, Object ExpressionSetConstraintObj, Insert the tab 'CML-4 ExpressionSetConstraintObj': ExpressionSetId = model Id (9QL…), ReferenceObjectId = product AIR2 Id (01t…), ConstraintModelTag = AirliteAIR2, ConstraintModelTagType = Type. Then refresh the builder and continue.</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
           <t>How a working model (ECO) is linked:
 SELECT Id, ExpressionSet.Name, ReferenceObjectId, ReferenceObject.Name, ConstraintModelTag, ConstraintModelTagType FROM ExpressionSetConstraintObj WHERE ExpressionSet.Name LIKE '%ECO%'
-Model Id:
+Model Id (9QL…):
 SELECT Id, Name FROM ExpressionSet WHERE Name LIKE '%AIR2%'
 Product Id:
 SELECT Id, Name FROM Product2 WHERE ProductCode = 'AIR2'</t>
@@ -2490,6 +2491,70 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ExpressionSetId</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ReferenceObjectId</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>ConstraintModelTag</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>ConstraintModelTagType</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>9QLAP000004prb34AA</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>&lt;Product2 Id 01t…&gt;</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>AirliteAIR2</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2559,7 +2624,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Inspector workbook: keep sheet names within Excel's 31-char limit
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D8YckfAx7oSp47X8zmY1mN
</commit_message>
<xml_diff>
--- a/OneDrive_2026-09-29/Claude RCA Product/10-airlite2-product-template/Airlite2_RCA_Import_Inspector.xlsx
+++ b/OneDrive_2026-09-29/Claude RCA Product/10-airlite2-product-template/Airlite2_RCA_Import_Inspector.xlsx
@@ -18,7 +18,7 @@
     <sheet name="08 ProductClassificationAttr" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="08 RETRY (failed rows)" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="09 ProductCategoryProduct" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="CML-4 ExpressionSetConstraintObj" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="CML-4 ExpressionSetConstrObj" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="10 PricebookEntry" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="11 Attribute_Pricing__c" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
@@ -762,7 +762,7 @@
       <c r="C14" s="2" t="inlineStr"/>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>REQUIRED before activation (else: 'We couldn't find any associations for constraint version 9QL…'). Not done in the Constraint Builder UI ('New Type' only adds a CML type; 'Add Labels' is unrelated). Inspector → Data Import, Object ExpressionSetConstraintObj, Insert the tab 'CML-4 ExpressionSetConstraintObj': ExpressionSetId = model Id (9QL…), ReferenceObjectId = product AIR2 Id (01t…), ConstraintModelTag = AirliteAIR2, ConstraintModelTagType = Type. Then refresh the builder and continue.</t>
+          <t>REQUIRED before activation (else: 'We couldn't find any associations for constraint version 9QL…'). Not done in the Constraint Builder UI ('New Type' only adds a CML type; 'Add Labels' is unrelated). Inspector → Data Import, Object ExpressionSetConstraintObj, Insert the tab 'CML-4 ExpressionSetConstrObj': ExpressionSetId = model Id (9QL…), ReferenceObjectId = product AIR2 Id (01t…), ConstraintModelTag = AirliteAIR2, ConstraintModelTagType = Type. Then refresh the builder and continue.</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Airlite2: CML-4 association row filled with model and product Ids
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D8YckfAx7oSp47X8zmY1mN
</commit_message>
<xml_diff>
--- a/OneDrive_2026-09-29/Claude RCA Product/10-airlite2-product-template/Airlite2_RCA_Import_Inspector.xlsx
+++ b/OneDrive_2026-09-29/Claude RCA Product/10-airlite2-product-template/Airlite2_RCA_Import_Inspector.xlsx
@@ -2523,14 +2523,14 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>9QLAP000004prb34AA</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>&lt;Product2 Id 01t…&gt;</t>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>01tAP00000UbUSUYA3</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Skill: PricebookEntry (price 0 placeholder) is required before testing on a quote
Tab 10 moves before TEST: without an active entry in the quote's price book and
currency the product does not appear in the product picker. Builder emits a
standard + quote price book row, the queries to find them, and the order
01-09 -> CML -> 10 -> TEST -> 11. Airlite2 workbook rebuilt (AIR2 Id filled).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D8YckfAx7oSp47X8zmY1mN
</commit_message>
<xml_diff>
--- a/OneDrive_2026-09-29/Claude RCA Product/10-airlite2-product-template/Airlite2_RCA_Import_Inspector.xlsx
+++ b/OneDrive_2026-09-29/Claude RCA Product/10-airlite2-product-template/Airlite2_RCA_Import_Inspector.xlsx
@@ -817,47 +817,53 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>TEST – Quote</t>
+          <t>10 PricebookEntry</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Quote</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr"/>
+          <t>Insert (price 0 placeholder)</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Create a quote, add the product, configure. Check: every attribute shows, dropdown values are right, invalid combinations are blocked with the rule message, calculated outputs fill in. Reference configuration: AIR2, Width 1200, Length 2100, Installation A0, Wind baffle WM → Av 2.52 m², Aa 1.42 m²</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr"/>
+          <t>REQUIRED before TEST: a product only appears in a quote's product picker with an active entry in the quote's price book and currency. Load now with UnitPrice 0, update when factory prices arrive. Standard Price Book row first (Salesforce requires it), then the quote's price book (skip row 2 if that is the standard one). One pair per currency the quotes use – copy the pattern of a similar product (query on Import Steps).</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Price books (standard + active):
+SELECT Id, Name, IsStandard, IsActive FROM Pricebook2 WHERE IsActive = true OR IsStandard = true
+Price book + currency of recent quotes:
+SELECT Id, Name, Pricebook2Id, Pricebook2.Name, CurrencyIsoCode FROM Quote ORDER BY CreatedDate DESC LIMIT 5
+Pattern of a similar product:
+SELECT Pricebook2.Name, Pricebook2.IsStandard, CurrencyIsoCode, UnitPrice, IsActive, UseStandardPrice FROM PricebookEntry WHERE Product2.ProductCode = '&lt;similar product code&gt;'
+Check after import:
+SELECT Pricebook2.Name, CurrencyIsoCode, UnitPrice, IsActive FROM PricebookEntry WHERE Product2.ProductCode = 'AIR2'</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>10 PricebookEntry</t>
+          <t>TEST – Quote</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Insert – LATER</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>Quote</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr"/>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Skip until the factory supplies prices. Standard Price Book entry first, then the KLAW price book.</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Pricebook2Id:
-SELECT Id, Name, IsStandard FROM Pricebook2 WHERE IsActive = true</t>
-        </is>
-      </c>
+          <t>Create a quote, add the product, configure. Check: every attribute shows, dropdown values are right, invalid combinations are blocked with the rule message, calculated outputs fill in. Reference configuration: AIR2, Width 1200, Length 2100, Installation A0, Wind baffle WM → Av 2.52 m², Aa 1.42 m²</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2555,7 +2561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2563,6 +2569,7 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2591,6 +2598,11 @@
           <t>CurrencyIsoCode</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>UseStandardPrice</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -2598,14 +2610,14 @@
           <t>&lt;Standard Price Book Id&gt;</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>&lt;Product2 Id&gt;</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>&lt;price&gt;</t>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>01tAP00000UbUSUYA3</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -2616,6 +2628,43 @@
       <c r="E2" s="3" t="inlineStr">
         <is>
           <t>EUR</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>&lt;Quote's price book Id&gt;</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>01tAP00000UbUSUYA3</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>false</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record the org's two price book Ids as defaults for tab 10
01s0Y000004WPyFQAW (standard, first) and 01sAP000003qiEXYAY (quote price
book) in CLAUDE.md, SKILL.md, the import reference and the workbook builder
(--pricebooks to override). Airlite2 tab 10 fully filled.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D8YckfAx7oSp47X8zmY1mN
</commit_message>
<xml_diff>
--- a/OneDrive_2026-09-29/Claude RCA Product/10-airlite2-product-template/Airlite2_RCA_Import_Inspector.xlsx
+++ b/OneDrive_2026-09-29/Claude RCA Product/10-airlite2-product-template/Airlite2_RCA_Import_Inspector.xlsx
@@ -830,7 +830,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>REQUIRED before TEST: a product only appears in a quote's product picker with an active entry in the quote's price book and currency. Load now with UnitPrice 0, update when factory prices arrive. Standard Price Book row first (Salesforce requires it), then the quote's price book (skip row 2 if that is the standard one). One pair per currency the quotes use – copy the pattern of a similar product (query on Import Steps).</t>
+          <t>REQUIRED before TEST: a product only appears in a quote's product picker with an active entry in the quote's price book and currency. Load now with UnitPrice 0, update when factory prices arrive. Standard Price Book row first (Salesforce requires it), then the quote's price book. Org price books: 01s0Y000004WPyFQAW = Standard price book – first; 01sAP000003qiEXYAY = Quote price book – second. One pair per currency the quotes use – copy the pattern of a similar product (query on Import Steps).</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -2564,7 +2564,7 @@
   <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -2605,9 +2605,9 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>&lt;Standard Price Book Id&gt;</t>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>01s0Y000004WPyFQAW</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -2637,9 +2637,9 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>&lt;Quote's price book Id&gt;</t>
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>01sAP000003qiEXYAY</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">

</xml_diff>